<commit_message>
White Mask Varré | Add project organisation diagram; Add full name to da-author; Finish project management chapter (except project finish report); Add table calculations for total cost as well as put them into appendix; Theoretical part of thesis almost done
</commit_message>
<xml_diff>
--- a/Diplomarbeit/doc/Schaar/Tabellenberechnungen-Diagramme-Diplomarbeit-Schaar.xlsx
+++ b/Diplomarbeit/doc/Schaar/Tabellenberechnungen-Diagramme-Diplomarbeit-Schaar.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kiese\OneDrive\Dokumente\Schule\Diplomarbeit\Diplomarbeit_Tischkicker\Diplomarbeit\doc\Schaar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2637B0D-283B-44CF-829A-9101ACDD01F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39CB3D33-B327-4745-840F-0C898BE0BC68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{6E91DB90-8AB8-47FA-9925-F6AA49AB0963}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" firstSheet="1" activeTab="3" xr2:uid="{6E91DB90-8AB8-47FA-9925-F6AA49AB0963}"/>
   </bookViews>
   <sheets>
     <sheet name="Diagramm - Punkteverteilung MCs" sheetId="1" r:id="rId1"/>
     <sheet name="Berechnung - Vergleich MCs" sheetId="2" r:id="rId2"/>
     <sheet name="Diagramm - Vergleich MCs" sheetId="3" r:id="rId3"/>
+    <sheet name="Geschätzte Gesamtkosten - DA" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="42">
   <si>
     <t>Vergleichsbasis</t>
   </si>
@@ -117,6 +118,54 @@
   <si>
     <t>Gesamtpunktzahl</t>
   </si>
+  <si>
+    <t>Kosten - Hardware</t>
+  </si>
+  <si>
+    <t>Gesamtkosten/St.</t>
+  </si>
+  <si>
+    <t>Gesamtkosten (2 St.)</t>
+  </si>
+  <si>
+    <t>Filament</t>
+  </si>
+  <si>
+    <t>Menge</t>
+  </si>
+  <si>
+    <t>~4-5 kg</t>
+  </si>
+  <si>
+    <t>Kabel</t>
+  </si>
+  <si>
+    <t>Breadboard</t>
+  </si>
+  <si>
+    <t>USB-Hub</t>
+  </si>
+  <si>
+    <t>Kosten - Druck</t>
+  </si>
+  <si>
+    <t>Kostenstelle</t>
+  </si>
+  <si>
+    <t>Gesamtkosten (5 St.)</t>
+  </si>
+  <si>
+    <t>https://www.buchbinderei-dienbauer.at/</t>
+  </si>
+  <si>
+    <t>Kosten-Quelle für Binden der Arbeit:</t>
+  </si>
+  <si>
+    <t>Drucken + Binden der Arbeit</t>
+  </si>
+  <si>
+    <t>Geplante Gesamtkosten der Arbeit</t>
+  </si>
 </sst>
 </file>
 
@@ -126,7 +175,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -188,8 +237,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="14"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -244,8 +309,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="25">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -543,13 +614,102 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -592,6 +752,31 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="17" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -683,6 +868,63 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="7" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="7" fillId="10" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4123,10 +4365,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="33"/>
+      <c r="B1" s="48"/>
     </row>
     <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -4205,12 +4447,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="36"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="51"/>
     </row>
     <row r="2" spans="1:4" ht="38.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="18" t="s">
@@ -4304,177 +4546,177 @@
     </row>
     <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="10" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="39"/>
+      <c r="B10" s="53"/>
+      <c r="C10" s="53"/>
+      <c r="D10" s="54"/>
     </row>
     <row r="11" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="41"/>
-      <c r="D11" s="42"/>
+      <c r="C11" s="56"/>
+      <c r="D11" s="57"/>
     </row>
     <row r="12" spans="1:4" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="43">
+      <c r="B12" s="58">
         <v>21.6</v>
       </c>
-      <c r="C12" s="44"/>
-      <c r="D12" s="45"/>
+      <c r="C12" s="59"/>
+      <c r="D12" s="60"/>
     </row>
     <row r="13" spans="1:4" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="43">
+      <c r="B13" s="58">
         <v>16.600000000000001</v>
       </c>
-      <c r="C13" s="44"/>
-      <c r="D13" s="45"/>
+      <c r="C13" s="59"/>
+      <c r="D13" s="60"/>
     </row>
     <row r="14" spans="1:4" ht="31.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="43">
+      <c r="B14" s="58">
         <v>19.97</v>
       </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
+      <c r="C14" s="59"/>
+      <c r="D14" s="60"/>
     </row>
     <row r="15" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="46">
+      <c r="B15" s="61">
         <f>AVERAGE(B12:B14)</f>
         <v>19.39</v>
       </c>
-      <c r="C15" s="47"/>
-      <c r="D15" s="48"/>
+      <c r="C15" s="62"/>
+      <c r="D15" s="63"/>
     </row>
     <row r="16" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="17"/>
-      <c r="B16" s="49"/>
-      <c r="C16" s="49"/>
-      <c r="D16" s="50"/>
+      <c r="B16" s="64"/>
+      <c r="C16" s="64"/>
+      <c r="D16" s="65"/>
     </row>
     <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="51" t="s">
+      <c r="B17" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="52"/>
-      <c r="D17" s="53"/>
+      <c r="C17" s="67"/>
+      <c r="D17" s="68"/>
     </row>
     <row r="18" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="43">
+      <c r="B18" s="58">
         <v>13</v>
       </c>
-      <c r="C18" s="44"/>
-      <c r="D18" s="45"/>
+      <c r="C18" s="59"/>
+      <c r="D18" s="60"/>
     </row>
     <row r="19" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="43">
+      <c r="B19" s="58">
         <v>13.99</v>
       </c>
-      <c r="C19" s="44"/>
-      <c r="D19" s="45"/>
+      <c r="C19" s="59"/>
+      <c r="D19" s="60"/>
     </row>
     <row r="20" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="43">
+      <c r="B20" s="58">
         <v>11.9</v>
       </c>
-      <c r="C20" s="44"/>
-      <c r="D20" s="45"/>
+      <c r="C20" s="59"/>
+      <c r="D20" s="60"/>
     </row>
     <row r="21" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="57">
+      <c r="B21" s="72">
         <f>AVERAGE(B18:B20)</f>
         <v>12.963333333333333</v>
       </c>
-      <c r="C21" s="58"/>
-      <c r="D21" s="59"/>
+      <c r="C21" s="73"/>
+      <c r="D21" s="74"/>
     </row>
     <row r="22" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="17"/>
-      <c r="B22" s="49"/>
-      <c r="C22" s="49"/>
-      <c r="D22" s="50"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="65"/>
     </row>
     <row r="23" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="60" t="s">
+      <c r="B23" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="61"/>
-      <c r="D23" s="62"/>
+      <c r="C23" s="76"/>
+      <c r="D23" s="77"/>
     </row>
     <row r="24" spans="1:4" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A24" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="43">
+      <c r="B24" s="58">
         <v>7.6</v>
       </c>
-      <c r="C24" s="44"/>
-      <c r="D24" s="45"/>
+      <c r="C24" s="59"/>
+      <c r="D24" s="60"/>
     </row>
     <row r="25" spans="1:4" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="43">
+      <c r="B25" s="58">
         <v>8</v>
       </c>
-      <c r="C25" s="44"/>
-      <c r="D25" s="45"/>
+      <c r="C25" s="59"/>
+      <c r="D25" s="60"/>
     </row>
     <row r="26" spans="1:4" ht="31.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="43">
+      <c r="B26" s="58">
         <v>8.57</v>
       </c>
-      <c r="C26" s="44"/>
-      <c r="D26" s="45"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="60"/>
     </row>
     <row r="27" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="54">
+      <c r="B27" s="69">
         <f>AVERAGE(B24:B26)</f>
         <v>8.0566666666666666</v>
       </c>
-      <c r="C27" s="55"/>
-      <c r="D27" s="56"/>
+      <c r="C27" s="70"/>
+      <c r="D27" s="71"/>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -4522,4 +4764,220 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{206D83DB-2C3C-4D55-B5CA-837D1457F631}">
+  <dimension ref="B1:D23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="37.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:4" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="84" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="85"/>
+      <c r="D2" s="86"/>
+    </row>
+    <row r="3" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="35" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B4" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="44">
+        <f>4.5*24</f>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B5" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="23">
+        <v>1</v>
+      </c>
+      <c r="D5" s="45">
+        <v>12.96</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B6" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="37" t="str">
+        <f>"10-15"</f>
+        <v>10-15</v>
+      </c>
+      <c r="D6" s="45">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B7" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="38">
+        <v>1</v>
+      </c>
+      <c r="D7" s="45">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="42" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="33">
+        <v>1</v>
+      </c>
+      <c r="D8" s="46">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="39" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="40"/>
+      <c r="D9" s="41">
+        <f>SUM(D4:D8)</f>
+        <v>135.21</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="40"/>
+      <c r="D10" s="41">
+        <f>D9*2</f>
+        <v>270.42</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="2:4" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="84" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="85"/>
+      <c r="D12" s="86"/>
+    </row>
+    <row r="13" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="87" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" s="88"/>
+    </row>
+    <row r="14" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B14" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="89">
+        <v>45</v>
+      </c>
+      <c r="D14" s="90"/>
+    </row>
+    <row r="15" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="43" t="str">
+        <f>"- 38% Schülerrabatt"</f>
+        <v>- 38% Schülerrabatt</v>
+      </c>
+      <c r="C15" s="91">
+        <f>(C14*0.38)*(-1)</f>
+        <v>-17.100000000000001</v>
+      </c>
+      <c r="D15" s="92"/>
+    </row>
+    <row r="16" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="93">
+        <f>SUM(C14:D15)</f>
+        <v>27.9</v>
+      </c>
+      <c r="D16" s="94"/>
+    </row>
+    <row r="17" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="93">
+        <f>C16*5</f>
+        <v>139.5</v>
+      </c>
+      <c r="D17" s="94"/>
+    </row>
+    <row r="19" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B19" s="95" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="95"/>
+      <c r="D19" s="95"/>
+    </row>
+    <row r="20" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B20" s="96" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="96"/>
+      <c r="D20" s="96"/>
+    </row>
+    <row r="21" spans="2:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="22" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="78" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="79"/>
+      <c r="D22" s="82">
+        <f>SUM(D10,C17)</f>
+        <v>409.92</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="80"/>
+      <c r="C23" s="81"/>
+      <c r="D23" s="83"/>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B20:D20"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B20" r:id="rId1" xr:uid="{5C44A1FD-6BD2-4635-BDEA-1144E26EE6AC}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rakshasa | Fix small formatting error of an image; Write summary of thesis; Finalize project management and add project finalization report; Add title of Prof. Hutter to thanks; Change some minor parts in metadata.yaml and add table calculations for actual project cost; Remove unused protocol file; Remove temporary file from Presentations folder
</commit_message>
<xml_diff>
--- a/Diplomarbeit/doc/Schaar/Tabellenberechnungen-Diagramme-Diplomarbeit-Schaar.xlsx
+++ b/Diplomarbeit/doc/Schaar/Tabellenberechnungen-Diagramme-Diplomarbeit-Schaar.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kiese\OneDrive\Dokumente\Schule\Diplomarbeit\Diplomarbeit_Tischkicker\Diplomarbeit\doc\Schaar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39CB3D33-B327-4745-840F-0C898BE0BC68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6568C0FF-5C18-47B9-8678-9BBEA4BEFB01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" firstSheet="1" activeTab="3" xr2:uid="{6E91DB90-8AB8-47FA-9925-F6AA49AB0963}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" firstSheet="2" activeTab="4" xr2:uid="{6E91DB90-8AB8-47FA-9925-F6AA49AB0963}"/>
   </bookViews>
   <sheets>
     <sheet name="Diagramm - Punkteverteilung MCs" sheetId="1" r:id="rId1"/>
     <sheet name="Berechnung - Vergleich MCs" sheetId="2" r:id="rId2"/>
     <sheet name="Diagramm - Vergleich MCs" sheetId="3" r:id="rId3"/>
     <sheet name="Geschätzte Gesamtkosten - DA" sheetId="4" r:id="rId4"/>
+    <sheet name="Tatsächliche Gesamtkosten - DA" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="46">
   <si>
     <t>Vergleichsbasis</t>
   </si>
@@ -165,6 +166,18 @@
   </si>
   <si>
     <t>Geplante Gesamtkosten der Arbeit</t>
+  </si>
+  <si>
+    <t>Raspberry Pi 4 Model B</t>
+  </si>
+  <si>
+    <t>Filament in kg</t>
+  </si>
+  <si>
+    <t>HP 125 Wired Mouse (von Schule)</t>
+  </si>
+  <si>
+    <t>Tatsächliche Gesamtkosten der Arbeit</t>
   </si>
 </sst>
 </file>
@@ -870,6 +883,15 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -886,15 +908,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="7" fillId="10" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4779,11 +4792,11 @@
   <sheetData>
     <row r="1" spans="2:4" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:4" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="84" t="s">
+      <c r="B2" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="85"/>
-      <c r="D2" s="86"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="80"/>
     </row>
     <row r="3" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="32" t="s">
@@ -4875,11 +4888,11 @@
     </row>
     <row r="11" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="12" spans="2:4" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="84" t="s">
+      <c r="B12" s="78" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="85"/>
-      <c r="D12" s="86"/>
+      <c r="C12" s="79"/>
+      <c r="D12" s="80"/>
     </row>
     <row r="13" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="32" t="s">
@@ -4946,19 +4959,19 @@
     </row>
     <row r="21" spans="2:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="22" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="78" t="s">
+      <c r="B22" s="81" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="79"/>
-      <c r="D22" s="82">
+      <c r="C22" s="82"/>
+      <c r="D22" s="85">
         <f>SUM(D10,C17)</f>
         <v>409.92</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="80"/>
-      <c r="C23" s="81"/>
-      <c r="D23" s="83"/>
+      <c r="B23" s="83"/>
+      <c r="C23" s="84"/>
+      <c r="D23" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -4980,4 +4993,197 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2347381E-D62B-4EAF-8043-11B1D254A222}">
+  <dimension ref="B1:D21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:4" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="78" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="79"/>
+      <c r="D2" s="80"/>
+    </row>
+    <row r="3" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="35" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B4" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="36">
+        <v>3.7</v>
+      </c>
+      <c r="D4" s="44">
+        <f>C4*22.99</f>
+        <v>85.063000000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B5" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="23">
+        <v>1</v>
+      </c>
+      <c r="D5" s="45">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="38">
+        <v>4</v>
+      </c>
+      <c r="D6" s="45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="39" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="40"/>
+      <c r="D7" s="41">
+        <f>SUM(D4:D6)</f>
+        <v>125.063</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="40"/>
+      <c r="D8" s="41">
+        <f>D7*2</f>
+        <v>250.126</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="2:4" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="78" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="79"/>
+      <c r="D10" s="80"/>
+    </row>
+    <row r="11" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="87" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="88"/>
+    </row>
+    <row r="12" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B12" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="89">
+        <v>45</v>
+      </c>
+      <c r="D12" s="90"/>
+    </row>
+    <row r="13" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="43" t="str">
+        <f>"- 38% Schülerrabatt"</f>
+        <v>- 38% Schülerrabatt</v>
+      </c>
+      <c r="C13" s="91">
+        <f>(C12*0.38)*(-1)</f>
+        <v>-17.100000000000001</v>
+      </c>
+      <c r="D13" s="92"/>
+    </row>
+    <row r="14" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="93">
+        <f>SUM(C12:D13)</f>
+        <v>27.9</v>
+      </c>
+      <c r="D14" s="94"/>
+    </row>
+    <row r="15" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="93">
+        <f>C14*5</f>
+        <v>139.5</v>
+      </c>
+      <c r="D15" s="94"/>
+    </row>
+    <row r="17" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B17" s="95" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="95"/>
+      <c r="D17" s="95"/>
+    </row>
+    <row r="18" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B18" s="96" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="96"/>
+      <c r="D18" s="96"/>
+    </row>
+    <row r="19" spans="2:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="20" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="81" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="82"/>
+      <c r="D20" s="85">
+        <f>SUM(D8,C15)</f>
+        <v>389.62599999999998</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="83"/>
+      <c r="C21" s="84"/>
+      <c r="D21" s="86"/>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B20:C21"/>
+    <mergeCell ref="D20:D21"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B18" r:id="rId1" xr:uid="{FA696D5D-EEB4-4692-8E9A-9CA2B06772A5}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>